<commit_message>
Update Strava data and site
</commit_message>
<xml_diff>
--- a/data/activities_log.xlsx
+++ b/data/activities_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,6 +451,33 @@
         <is>
           <t>elapsed_time</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Théo|D.|Afternoon Run|1000.0|360|360</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ThéoD.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Afternoon Run</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F2" t="n">
+        <v>360</v>
+      </c>
+      <c r="G2" t="n">
+        <v>360</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Normalize Strava member matching
</commit_message>
<xml_diff>
--- a/data/activities_log.xlsx
+++ b/data/activities_log.xlsx
@@ -459,7 +459,11 @@
           <t>Théo|D.|Afternoon Run|1000.0|360|360</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Team 1</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>ThéoD.</t>

</xml_diff>

<commit_message>
Restore missing AntoL activity
</commit_message>
<xml_diff>
--- a/data/activities_log.xlsx
+++ b/data/activities_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G187"/>
+  <dimension ref="A1:G188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6191,6 +6191,37 @@
         <v>3738</v>
       </c>
     </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Anto|L.|Afternoon Run|10003.5|3429|3583</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>MAMA l'équipe</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>AntoL.</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Afternoon Run</t>
+        </is>
+      </c>
+      <c r="E188" t="n">
+        <v>10003.5</v>
+      </c>
+      <c r="F188" t="n">
+        <v>3429</v>
+      </c>
+      <c r="G188" t="n">
+        <v>3583</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Preserve activity history and restore validated activities
</commit_message>
<xml_diff>
--- a/data/activities_log.xlsx
+++ b/data/activities_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G188"/>
+  <dimension ref="A1:G211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6206,6 +6206,719 @@
         <v>4783</v>
       </c>
     </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>manual|Agathe|M.|Night Run|5667.6|2415|2460</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>MAMA l'équipe</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>AgatheM.</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Night Run</t>
+        </is>
+      </c>
+      <c r="E189" t="n">
+        <v>5667.6</v>
+      </c>
+      <c r="F189" t="n">
+        <v>2415</v>
+      </c>
+      <c r="G189" t="n">
+        <v>2460</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>manual|Alejandra|S.|Que calorrrr|5097.7|1754|2957</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Croquetas</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>AlejandraS.</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Que calorrrr</t>
+        </is>
+      </c>
+      <c r="E190" t="n">
+        <v>5097.7</v>
+      </c>
+      <c r="F190" t="n">
+        <v>1754</v>
+      </c>
+      <c r="G190" t="n">
+        <v>2957</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>manual|Ben|B.|Course à pied de nuit|10124.0|3124|3196</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Esiee en sueur</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>BenB.</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Course à pied de nuit</t>
+        </is>
+      </c>
+      <c r="E191" t="n">
+        <v>10124</v>
+      </c>
+      <c r="F191" t="n">
+        <v>3124</v>
+      </c>
+      <c r="G191" t="n">
+        <v>3196</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>manual|Celestin|L.|7 x 1,6km seuil + 0,8km recup|22275.0|8443|9091</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Les Loulous</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>CelestinL.</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>7 x 1,6km seuil + 0,8km recup</t>
+        </is>
+      </c>
+      <c r="E192" t="n">
+        <v>22275</v>
+      </c>
+      <c r="F192" t="n">
+        <v>8443</v>
+      </c>
+      <c r="G192" t="n">
+        <v>9091</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>manual|Clément|G.|Evening Run|10111.6|3233|3400</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Esiee en sueur</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>ClémentG.</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Evening Run</t>
+        </is>
+      </c>
+      <c r="E193" t="n">
+        <v>10111.6</v>
+      </c>
+      <c r="F193" t="n">
+        <v>3233</v>
+      </c>
+      <c r="G193" t="n">
+        <v>3400</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>manual|Enzo|L.|Course à pied de nuit|1345.1|767|1006</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Les Loulous</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>EnzoL.</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Course à pied de nuit</t>
+        </is>
+      </c>
+      <c r="E194" t="n">
+        <v>1345.1</v>
+      </c>
+      <c r="F194" t="n">
+        <v>767</v>
+      </c>
+      <c r="G194" t="n">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>manual|Enzo|L.|Course à pied le soir|3263.4|1403|4714</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Les Loulous</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>EnzoL.</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Course à pied le soir</t>
+        </is>
+      </c>
+      <c r="E195" t="n">
+        <v>3263.4</v>
+      </c>
+      <c r="F195" t="n">
+        <v>1403</v>
+      </c>
+      <c r="G195" t="n">
+        <v>4714</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>manual|Esteban|B.|Team 67|13670.5|4839|4993</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>67 kilometers</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>EstebanB.</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Team 67</t>
+        </is>
+      </c>
+      <c r="E196" t="n">
+        <v>13670.5</v>
+      </c>
+      <c r="F196" t="n">
+        <v>4839</v>
+      </c>
+      <c r="G196" t="n">
+        <v>4993</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>manual|Ethan|S.|Course à pied de nuit|660.9|211|260</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Esiee en sueur</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>EthanS.</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Course à pied de nuit</t>
+        </is>
+      </c>
+      <c r="E197" t="n">
+        <v>660.9</v>
+      </c>
+      <c r="F197" t="n">
+        <v>211</v>
+      </c>
+      <c r="G197" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>manual|Lyne|V.|J-3 : Sortie de recup|4399.5|2114|2173</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Les asiats</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>LyneV.</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>J-3 : Sortie de recup</t>
+        </is>
+      </c>
+      <c r="E198" t="n">
+        <v>4399.5</v>
+      </c>
+      <c r="F198" t="n">
+        <v>2114</v>
+      </c>
+      <c r="G198" t="n">
+        <v>2173</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>manual|Matheo|D.|Team 67|6697.0|2430|2435</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>67 kilometers</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>MatheoD.</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Team 67</t>
+        </is>
+      </c>
+      <c r="E199" t="n">
+        <v>6697</v>
+      </c>
+      <c r="F199" t="n">
+        <v>2430</v>
+      </c>
+      <c r="G199" t="n">
+        <v>2435</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>manual|Mathis|G.|Course soirée chill|5936.5|2432|2498</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>MAMA l'équipe</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>MathisG.</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Course soirée chill</t>
+        </is>
+      </c>
+      <c r="E200" t="n">
+        <v>5936.5</v>
+      </c>
+      <c r="F200" t="n">
+        <v>2432</v>
+      </c>
+      <c r="G200" t="n">
+        <v>2498</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>manual|Mederic|-.|Course à pied de nuit|7042.6|2515|3087</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>MAMA l'équipe</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Mederic-.</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Course à pied de nuit</t>
+        </is>
+      </c>
+      <c r="E201" t="n">
+        <v>7042.6</v>
+      </c>
+      <c r="F201" t="n">
+        <v>2515</v>
+      </c>
+      <c r="G201" t="n">
+        <v>3087</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>manual|Romain|P.|Marquage du territoire pour assouvir la dominance|14140.2|5775|5877</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Les Teambrés</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>RomainP.</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Marquage du territoire pour assouvir la dominance</t>
+        </is>
+      </c>
+      <c r="E202" t="n">
+        <v>14140.2</v>
+      </c>
+      <c r="F202" t="n">
+        <v>5775</v>
+      </c>
+      <c r="G202" t="n">
+        <v>5877</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>manual|Samy|A.|Échauffement je crois|2005.5|914|990</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Croquetas</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>SamyA.</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Échauffement je crois</t>
+        </is>
+      </c>
+      <c r="E203" t="n">
+        <v>2005.5</v>
+      </c>
+      <c r="F203" t="n">
+        <v>914</v>
+      </c>
+      <c r="G203" t="n">
+        <v>990</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>manual|Steve|D.|Course à pied de nuit|1144.6|733|977</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Akatsuki</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>SteveD.</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Course à pied de nuit</t>
+        </is>
+      </c>
+      <c r="E204" t="n">
+        <v>1144.6</v>
+      </c>
+      <c r="F204" t="n">
+        <v>733</v>
+      </c>
+      <c r="G204" t="n">
+        <v>977</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>manual|Thibault|L.|Course à pied le soir|5398.5|2234|2319</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Les Loulous</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>ThibaultL.</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Course à pied le soir</t>
+        </is>
+      </c>
+      <c r="E205" t="n">
+        <v>5398.5</v>
+      </c>
+      <c r="F205" t="n">
+        <v>2234</v>
+      </c>
+      <c r="G205" t="n">
+        <v>2319</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>manual|Théo|D.|Course VS 1/7|5023.9|2147|2171</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Les mixés</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>ThéoD.</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Course VS 1/7</t>
+        </is>
+      </c>
+      <c r="E206" t="n">
+        <v>5023.9</v>
+      </c>
+      <c r="F206" t="n">
+        <v>2147</v>
+      </c>
+      <c r="G206" t="n">
+        <v>2171</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>manual|Timothée|P.|Course à pied en soirée|12601.8|3707|6615</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Lukético</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>TimothéeP.</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Course à pied en soirée</t>
+        </is>
+      </c>
+      <c r="E207" t="n">
+        <v>12601.8</v>
+      </c>
+      <c r="F207" t="n">
+        <v>3707</v>
+      </c>
+      <c r="G207" t="n">
+        <v>6615</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>manual|Usman|S.|Vamos Team 67|10671.7|3654|3754</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>67 kilometers</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>UsmanS.</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Vamos Team 67</t>
+        </is>
+      </c>
+      <c r="E208" t="n">
+        <v>10671.7</v>
+      </c>
+      <c r="F208" t="n">
+        <v>3654</v>
+      </c>
+      <c r="G208" t="n">
+        <v>3754</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>manual|Valentin|C.|Team 67|15691.7|5971|6633</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>67 kilometers</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>ValentinC.</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Team 67</t>
+        </is>
+      </c>
+      <c r="E209" t="n">
+        <v>15691.7</v>
+      </c>
+      <c r="F209" t="n">
+        <v>5971</v>
+      </c>
+      <c r="G209" t="n">
+        <v>6633</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>manual|VlI|B.|Course à pied de nuit|15769.6|6133|7816</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Croquetas</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>VlIB.</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Course à pied de nuit</t>
+        </is>
+      </c>
+      <c r="E210" t="n">
+        <v>15769.6</v>
+      </c>
+      <c r="F210" t="n">
+        <v>6133</v>
+      </c>
+      <c r="G210" t="n">
+        <v>7816</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>manual|s|G.|Course à pied le soir|6194.4|2240|2287</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Les mixés</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>sG.</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Course à pied le soir</t>
+        </is>
+      </c>
+      <c r="E211" t="n">
+        <v>6194.4</v>
+      </c>
+      <c r="F211" t="n">
+        <v>2240</v>
+      </c>
+      <c r="G211" t="n">
+        <v>2287</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>